<commit_message>
docs(fix): re fix, avancement sprint 2 déja marqué comme fini
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-09-sprint-backlog-v3.0.xlsx
+++ b/docs/cadrage/equipe-09-sprint-backlog-v3.0.xlsx
@@ -14,9 +14,7 @@
     <sheet name="Burndown Sprint 1" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Sprint 2" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Burndown Sprint 2" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Sprint 3" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Burndown Sprint 3" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="Auto-évaluation" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Auto-évaluation" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="185">
   <si>
     <t xml:space="preserve">A</t>
   </si>
@@ -430,6 +428,9 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">Todo</t>
+  </si>
+  <si>
     <t xml:space="preserve">T-03.2</t>
   </si>
   <si>
@@ -515,18 +516,6 @@
   </si>
   <si>
     <t xml:space="preserve">13h00, Avant clôture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SPRINT BACKLOG : SPRINT 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mardi 30/06/2026, 14h00 à 18h00 (4 h)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BURNDOWN : SPRINT 3</t>
   </si>
   <si>
     <t xml:space="preserve">✅ Grille d'auto-évaluation</t>
@@ -621,7 +610,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -839,12 +828,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF1E1B4B"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color theme="1"/>
       <name val="Cambria"/>
       <family val="0"/>
@@ -971,7 +954,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="51">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1165,10 +1148,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="20" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2371,10 +2350,10 @@
         <v>1</v>
       </c>
       <c r="F20" s="43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" s="42" t="s">
-        <v>59</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2382,10 +2361,10 @@
         <v>130</v>
       </c>
       <c r="B21" s="44" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C21" s="40" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D21" s="42" t="s">
         <v>58</v>
@@ -2394,10 +2373,10 @@
         <v>1</v>
       </c>
       <c r="F21" s="43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" s="42" t="s">
-        <v>59</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2405,10 +2384,10 @@
         <v>130</v>
       </c>
       <c r="B22" s="44" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C22" s="45" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D22" s="42" t="s">
         <v>73</v>
@@ -2417,10 +2396,10 @@
         <v>1</v>
       </c>
       <c r="F22" s="43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22" s="42" t="s">
-        <v>59</v>
+        <v>133</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2428,10 +2407,10 @@
         <v>130</v>
       </c>
       <c r="B23" s="44" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C23" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D23" s="42" t="s">
         <v>62</v>
@@ -2440,10 +2419,10 @@
         <v>1</v>
       </c>
       <c r="F23" s="43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" s="42" t="s">
-        <v>59</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2451,22 +2430,22 @@
         <v>130</v>
       </c>
       <c r="B24" s="44" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C24" s="46" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D24" s="42" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E24" s="43" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" s="42" t="s">
-        <v>59</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2474,10 +2453,10 @@
         <v>130</v>
       </c>
       <c r="B25" s="44" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C25" s="40" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D25" s="42" t="s">
         <v>67</v>
@@ -2486,21 +2465,21 @@
         <v>1</v>
       </c>
       <c r="F25" s="43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" s="42" t="s">
-        <v>59</v>
+        <v>133</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B26" s="47" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C26" s="47" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D26" s="47" t="s">
         <v>58</v>
@@ -2509,21 +2488,21 @@
         <v>1</v>
       </c>
       <c r="F26" s="47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G26" s="48" t="s">
-        <v>59</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B27" s="47" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C27" s="47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D27" s="47" t="s">
         <v>73</v>
@@ -2532,21 +2511,21 @@
         <v>2</v>
       </c>
       <c r="F27" s="47" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G27" s="48" t="s">
-        <v>59</v>
+        <v>133</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B28" s="47" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C28" s="47" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D28" s="47" t="s">
         <v>62</v>
@@ -2555,44 +2534,44 @@
         <v>2</v>
       </c>
       <c r="F28" s="47" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G28" s="48" t="s">
-        <v>59</v>
+        <v>133</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B29" s="47" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C29" s="47" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D29" s="47" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E29" s="47" t="n">
         <v>2</v>
       </c>
       <c r="F29" s="47" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G29" s="48" t="s">
-        <v>59</v>
+        <v>133</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B30" s="47" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C30" s="47" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D30" s="47" t="s">
         <v>67</v>
@@ -2601,10 +2580,10 @@
         <v>2</v>
       </c>
       <c r="F30" s="47" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G30" s="48" t="s">
-        <v>59</v>
+        <v>133</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2618,7 +2597,7 @@
         <v>15</v>
       </c>
       <c r="F31" s="33" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G31" s="34"/>
     </row>
@@ -2686,7 +2665,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2727,14 +2706,12 @@
     </row>
     <row r="8" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="38" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B8" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="C8" s="39" t="n">
-        <v>15</v>
-      </c>
+      <c r="C8" s="39"/>
       <c r="D8" s="39" t="n">
         <v>0</v>
       </c>
@@ -2744,48 +2721,42 @@
     </row>
     <row r="9" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="38" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B9" s="39" t="n">
         <v>10</v>
       </c>
-      <c r="C9" s="39" t="n">
-        <v>11</v>
-      </c>
+      <c r="C9" s="39"/>
       <c r="D9" s="39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="38" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B10" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="39" t="n">
-        <v>6</v>
-      </c>
+      <c r="C10" s="39"/>
       <c r="D10" s="39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B11" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="39" t="n">
-        <v>0</v>
-      </c>
+      <c r="C11" s="39"/>
       <c r="D11" s="39" t="n">
         <v>0</v>
       </c>
@@ -2855,633 +2826,6 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="11"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="38.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="36.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="48.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="49" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="s">
-        <v>45</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="22" t="s">
-        <v>47</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="B19" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="C19" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="D19" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="E19" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="F19" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="G19" s="23" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="B20" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="C20" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="D20" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="E20" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="25" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="B21" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="C21" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="D21" s="25" t="s">
-        <v>62</v>
-      </c>
-      <c r="E21" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="25" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="B22" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="C22" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="D22" s="25" t="s">
-        <v>62</v>
-      </c>
-      <c r="E22" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="F22" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="25" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23" s="24" t="s">
-        <v>65</v>
-      </c>
-      <c r="C23" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="D23" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="E23" s="26" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="25" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="B24" s="27" t="s">
-        <v>69</v>
-      </c>
-      <c r="C24" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="D24" s="28" t="s">
-        <v>58</v>
-      </c>
-      <c r="E24" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="F24" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="28" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="B25" s="27" t="s">
-        <v>71</v>
-      </c>
-      <c r="C25" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="D25" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="E25" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="28" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="B26" s="27" t="s">
-        <v>74</v>
-      </c>
-      <c r="C26" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="D26" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="E26" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="28" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="B27" s="27" t="s">
-        <v>76</v>
-      </c>
-      <c r="C27" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="D27" s="28" t="s">
-        <v>78</v>
-      </c>
-      <c r="E27" s="29" t="n">
-        <v>3</v>
-      </c>
-      <c r="F27" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="28" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="B28" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="C28" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="D28" s="28" t="s">
-        <v>67</v>
-      </c>
-      <c r="E28" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="28" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="30"/>
-      <c r="B29" s="30"/>
-      <c r="C29" s="31" t="s">
-        <v>81</v>
-      </c>
-      <c r="D29" s="31"/>
-      <c r="E29" s="32"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="31"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="33" t="s">
-        <v>82</v>
-      </c>
-      <c r="B30" s="34"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="34"/>
-      <c r="E30" s="33" t="n">
-        <v>16</v>
-      </c>
-      <c r="F30" s="33" t="n">
-        <v>16</v>
-      </c>
-      <c r="G30" s="34"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="36" t="s">
-        <v>59</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="37" t="s">
-        <v>85</v>
-      </c>
-      <c r="B34" s="10" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="22" t="s">
-        <v>87</v>
-      </c>
-      <c r="B35" s="10" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="B36" s="10" t="s">
-        <v>89</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="35"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>98</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="38" t="s">
-        <v>101</v>
-      </c>
-      <c r="B8" s="39" t="n">
-        <v>16</v>
-      </c>
-      <c r="C8" s="39" t="n">
-        <v>16</v>
-      </c>
-      <c r="D8" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="19" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="38" t="s">
-        <v>103</v>
-      </c>
-      <c r="B9" s="39" t="n">
-        <v>11</v>
-      </c>
-      <c r="C9" s="39" t="n">
-        <v>12</v>
-      </c>
-      <c r="D9" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="19" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="38" t="s">
-        <v>105</v>
-      </c>
-      <c r="B10" s="39" t="n">
-        <v>6</v>
-      </c>
-      <c r="C10" s="39" t="n">
-        <v>7</v>
-      </c>
-      <c r="D10" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="19" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="38" t="s">
-        <v>107</v>
-      </c>
-      <c r="B11" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="39" t="n">
-        <v>3</v>
-      </c>
-      <c r="D11" s="39" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" s="19" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="38" t="s">
-        <v>109</v>
-      </c>
-      <c r="B12" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="19" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
-        <v>118</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="22" t="s">
-        <v>120</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>121</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
   <dimension ref="A2:D15"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -3493,126 +2837,126 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="10" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23"/>
       <c r="B5" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="49" t="s">
         <v>168</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C6" s="50" t="s">
         <v>169</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D6" s="49" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="50" t="s">
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="49" t="s">
         <v>171</v>
       </c>
-      <c r="C6" s="51" t="s">
+      <c r="C7" s="50" t="s">
+        <v>169</v>
+      </c>
+      <c r="D7" s="49" t="s">
         <v>172</v>
       </c>
-      <c r="D6" s="50" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="49" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="50" t="s">
+      <c r="C8" s="50" t="s">
+        <v>169</v>
+      </c>
+      <c r="D8" s="49" t="s">
         <v>174</v>
       </c>
-      <c r="C7" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="D7" s="50" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="49" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="50" t="s">
+      <c r="C9" s="50" t="s">
+        <v>169</v>
+      </c>
+      <c r="D9" s="49" t="s">
         <v>176</v>
       </c>
-      <c r="C8" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="D8" s="50" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="49" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="50" t="s">
+      <c r="C10" s="50" t="s">
+        <v>169</v>
+      </c>
+      <c r="D10" s="49"/>
+    </row>
+    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="49" t="s">
         <v>178</v>
       </c>
-      <c r="C9" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="D9" s="50" t="s">
+      <c r="C11" s="50" t="s">
+        <v>169</v>
+      </c>
+      <c r="D11" s="49" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="50" t="s">
+    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="49" t="s">
         <v>180</v>
       </c>
-      <c r="C10" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="D10" s="50"/>
-    </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="50" t="s">
+      <c r="C12" s="50" t="s">
+        <v>169</v>
+      </c>
+      <c r="D12" s="49"/>
+    </row>
+    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="49" t="s">
         <v>181</v>
       </c>
-      <c r="C11" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="D11" s="50" t="s">
+      <c r="C13" s="50" t="s">
+        <v>169</v>
+      </c>
+      <c r="D13" s="49"/>
+    </row>
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="49" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="50" t="s">
+      <c r="C14" s="50" t="s">
+        <v>169</v>
+      </c>
+      <c r="D14" s="49"/>
+    </row>
+    <row r="15" customFormat="false" ht="53.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="49" t="s">
         <v>183</v>
       </c>
-      <c r="C12" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="D12" s="50"/>
-    </row>
-    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="50" t="s">
+      <c r="C15" s="50" t="s">
+        <v>169</v>
+      </c>
+      <c r="D15" s="49" t="s">
         <v>184</v>
-      </c>
-      <c r="C13" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="D13" s="50"/>
-    </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="50" t="s">
-        <v>185</v>
-      </c>
-      <c r="C14" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="D14" s="50"/>
-    </row>
-    <row r="15" customFormat="false" ht="53.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="50" t="s">
-        <v>186</v>
-      </c>
-      <c r="C15" s="51" t="s">
-        <v>172</v>
-      </c>
-      <c r="D15" s="50" t="s">
-        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(fix): done sprint 2 oublié
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-09-sprint-backlog-v3.0.xlsx
+++ b/docs/cadrage/equipe-09-sprint-backlog-v3.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Garde" sheetId="1" state="visible" r:id="rId3"/>
@@ -430,9 +430,6 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Todo</t>
-  </si>
-  <si>
     <t xml:space="preserve">T-03.2</t>
   </si>
   <si>
@@ -543,6 +540,9 @@
   </si>
   <si>
     <t xml:space="preserve">Vérifier exposition Quiz.score + details[] (bon/mauvais) dans la réponse POST /api/quizzes/&lt;id&gt;/answer/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todo</t>
   </si>
   <si>
     <t xml:space="preserve">T-05.2</t>
@@ -1093,7 +1093,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="54">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1288,10 +1288,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="29" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -2508,7 +2504,7 @@
         <v>1</v>
       </c>
       <c r="G20" s="43" t="s">
-        <v>133</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2516,10 +2512,10 @@
         <v>130</v>
       </c>
       <c r="B21" s="45" t="s">
+        <v>133</v>
+      </c>
+      <c r="C21" s="41" t="s">
         <v>134</v>
-      </c>
-      <c r="C21" s="41" t="s">
-        <v>135</v>
       </c>
       <c r="D21" s="43" t="s">
         <v>58</v>
@@ -2531,7 +2527,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="43" t="s">
-        <v>133</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2539,10 +2535,10 @@
         <v>130</v>
       </c>
       <c r="B22" s="45" t="s">
+        <v>135</v>
+      </c>
+      <c r="C22" s="46" t="s">
         <v>136</v>
-      </c>
-      <c r="C22" s="46" t="s">
-        <v>137</v>
       </c>
       <c r="D22" s="43" t="s">
         <v>73</v>
@@ -2554,7 +2550,7 @@
         <v>1</v>
       </c>
       <c r="G22" s="43" t="s">
-        <v>133</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2562,10 +2558,10 @@
         <v>130</v>
       </c>
       <c r="B23" s="45" t="s">
+        <v>137</v>
+      </c>
+      <c r="C23" s="41" t="s">
         <v>138</v>
-      </c>
-      <c r="C23" s="41" t="s">
-        <v>139</v>
       </c>
       <c r="D23" s="43" t="s">
         <v>62</v>
@@ -2577,7 +2573,7 @@
         <v>1</v>
       </c>
       <c r="G23" s="43" t="s">
-        <v>133</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2585,14 +2581,14 @@
         <v>130</v>
       </c>
       <c r="B24" s="45" t="s">
+        <v>139</v>
+      </c>
+      <c r="C24" s="47" t="s">
         <v>140</v>
       </c>
-      <c r="C24" s="47" t="s">
+      <c r="D24" s="43" t="s">
         <v>141</v>
       </c>
-      <c r="D24" s="43" t="s">
-        <v>142</v>
-      </c>
       <c r="E24" s="44" t="n">
         <v>1</v>
       </c>
@@ -2600,7 +2596,7 @@
         <v>1</v>
       </c>
       <c r="G24" s="43" t="s">
-        <v>133</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2608,10 +2604,10 @@
         <v>130</v>
       </c>
       <c r="B25" s="45" t="s">
+        <v>142</v>
+      </c>
+      <c r="C25" s="41" t="s">
         <v>143</v>
-      </c>
-      <c r="C25" s="41" t="s">
-        <v>144</v>
       </c>
       <c r="D25" s="43" t="s">
         <v>67</v>
@@ -2623,18 +2619,18 @@
         <v>1</v>
       </c>
       <c r="G25" s="43" t="s">
-        <v>133</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="48" t="s">
+        <v>144</v>
+      </c>
+      <c r="B26" s="48" t="s">
         <v>145</v>
       </c>
-      <c r="B26" s="48" t="s">
+      <c r="C26" s="48" t="s">
         <v>146</v>
-      </c>
-      <c r="C26" s="48" t="s">
-        <v>147</v>
       </c>
       <c r="D26" s="48" t="s">
         <v>58</v>
@@ -2645,19 +2641,19 @@
       <c r="F26" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="G26" s="49" t="s">
-        <v>133</v>
+      <c r="G26" s="43" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="48" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B27" s="48" t="s">
+        <v>147</v>
+      </c>
+      <c r="C27" s="48" t="s">
         <v>148</v>
-      </c>
-      <c r="C27" s="48" t="s">
-        <v>149</v>
       </c>
       <c r="D27" s="48" t="s">
         <v>73</v>
@@ -2668,19 +2664,19 @@
       <c r="F27" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="G27" s="49" t="s">
-        <v>133</v>
+      <c r="G27" s="43" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="48" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B28" s="48" t="s">
+        <v>149</v>
+      </c>
+      <c r="C28" s="48" t="s">
         <v>150</v>
-      </c>
-      <c r="C28" s="48" t="s">
-        <v>151</v>
       </c>
       <c r="D28" s="48" t="s">
         <v>62</v>
@@ -2691,22 +2687,22 @@
       <c r="F28" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="49" t="s">
-        <v>133</v>
+      <c r="G28" s="43" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="48" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B29" s="48" t="s">
+        <v>151</v>
+      </c>
+      <c r="C29" s="48" t="s">
         <v>152</v>
       </c>
-      <c r="C29" s="48" t="s">
-        <v>153</v>
-      </c>
       <c r="D29" s="48" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E29" s="48" t="n">
         <v>2</v>
@@ -2714,19 +2710,19 @@
       <c r="F29" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="G29" s="49" t="s">
-        <v>133</v>
+      <c r="G29" s="43" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="48" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B30" s="48" t="s">
+        <v>153</v>
+      </c>
+      <c r="C30" s="48" t="s">
         <v>154</v>
-      </c>
-      <c r="C30" s="48" t="s">
-        <v>155</v>
       </c>
       <c r="D30" s="48" t="s">
         <v>67</v>
@@ -2737,8 +2733,8 @@
       <c r="F30" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="G30" s="49" t="s">
-        <v>133</v>
+      <c r="G30" s="43" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2820,7 +2816,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2861,7 +2857,7 @@
     </row>
     <row r="8" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="38" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B8" s="39" t="n">
         <v>15</v>
@@ -2878,7 +2874,7 @@
     </row>
     <row r="9" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="38" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B9" s="39" t="n">
         <v>10</v>
@@ -2890,12 +2886,12 @@
         <v>1</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="38" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B10" s="39" t="n">
         <v>5</v>
@@ -2907,12 +2903,12 @@
         <v>1</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="38" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B11" s="39" t="n">
         <v>0</v>
@@ -3002,7 +2998,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3018,7 +3014,7 @@
         <v>25</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="38.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3026,7 +3022,7 @@
         <v>27</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3050,7 +3046,7 @@
         <v>33</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="48.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3058,7 +3054,7 @@
         <v>35</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3133,325 +3129,325 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="45.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="49" t="s">
+        <v>167</v>
+      </c>
+      <c r="B20" s="49" t="s">
         <v>168</v>
       </c>
-      <c r="B20" s="50" t="s">
+      <c r="C20" s="49" t="s">
         <v>169</v>
       </c>
-      <c r="C20" s="50" t="s">
+      <c r="D20" s="49" t="s">
+        <v>58</v>
+      </c>
+      <c r="E20" s="49" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="49" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" s="49" t="s">
         <v>170</v>
       </c>
-      <c r="D20" s="50" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="49" t="s">
+        <v>167</v>
+      </c>
+      <c r="B21" s="49" t="s">
+        <v>171</v>
+      </c>
+      <c r="C21" s="49" t="s">
+        <v>172</v>
+      </c>
+      <c r="D21" s="49" t="s">
+        <v>62</v>
+      </c>
+      <c r="E21" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="49" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="49" t="s">
+        <v>167</v>
+      </c>
+      <c r="B22" s="49" t="s">
+        <v>173</v>
+      </c>
+      <c r="C22" s="49" t="s">
+        <v>174</v>
+      </c>
+      <c r="D22" s="49" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="49" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="49" t="s">
+        <v>167</v>
+      </c>
+      <c r="B23" s="49" t="s">
+        <v>175</v>
+      </c>
+      <c r="C23" s="49" t="s">
+        <v>176</v>
+      </c>
+      <c r="D23" s="49" t="s">
+        <v>141</v>
+      </c>
+      <c r="E23" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="49" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="49" t="s">
+        <v>167</v>
+      </c>
+      <c r="B24" s="49" t="s">
+        <v>177</v>
+      </c>
+      <c r="C24" s="49" t="s">
+        <v>178</v>
+      </c>
+      <c r="D24" s="49" t="s">
+        <v>67</v>
+      </c>
+      <c r="E24" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="49" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="50" t="s">
+        <v>179</v>
+      </c>
+      <c r="B25" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="C25" s="50" t="s">
+        <v>181</v>
+      </c>
+      <c r="D25" s="50" t="s">
+        <v>73</v>
+      </c>
+      <c r="E25" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="50" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="50" t="s">
+        <v>179</v>
+      </c>
+      <c r="B26" s="50" t="s">
+        <v>182</v>
+      </c>
+      <c r="C26" s="50" t="s">
+        <v>183</v>
+      </c>
+      <c r="D26" s="50" t="s">
         <v>58</v>
       </c>
-      <c r="E20" s="50" t="n">
+      <c r="E26" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="50" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="50" t="s">
+        <v>179</v>
+      </c>
+      <c r="B27" s="50" t="s">
+        <v>184</v>
+      </c>
+      <c r="C27" s="50" t="s">
+        <v>185</v>
+      </c>
+      <c r="D27" s="50" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="50" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="50" t="s">
+        <v>179</v>
+      </c>
+      <c r="B28" s="50" t="s">
+        <v>186</v>
+      </c>
+      <c r="C28" s="50" t="s">
+        <v>187</v>
+      </c>
+      <c r="D28" s="50" t="s">
+        <v>141</v>
+      </c>
+      <c r="E28" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="50" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="50" t="s">
+        <v>179</v>
+      </c>
+      <c r="B29" s="50" t="s">
+        <v>188</v>
+      </c>
+      <c r="C29" s="50" t="s">
+        <v>189</v>
+      </c>
+      <c r="D29" s="50" t="s">
+        <v>67</v>
+      </c>
+      <c r="E29" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="50" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="52.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="51" t="s">
+        <v>190</v>
+      </c>
+      <c r="B30" s="51" t="s">
+        <v>191</v>
+      </c>
+      <c r="C30" s="51" t="s">
+        <v>192</v>
+      </c>
+      <c r="D30" s="51" t="s">
+        <v>73</v>
+      </c>
+      <c r="E30" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="F20" s="50" t="n">
+      <c r="F30" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="G20" s="50" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="50" t="s">
-        <v>168</v>
-      </c>
-      <c r="B21" s="50" t="s">
-        <v>171</v>
-      </c>
-      <c r="C21" s="50" t="s">
-        <v>172</v>
-      </c>
-      <c r="D21" s="50" t="s">
+      <c r="G30" s="51" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="51" t="s">
+        <v>190</v>
+      </c>
+      <c r="B31" s="51" t="s">
+        <v>193</v>
+      </c>
+      <c r="C31" s="51" t="s">
+        <v>194</v>
+      </c>
+      <c r="D31" s="51" t="s">
         <v>62</v>
       </c>
-      <c r="E21" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="50" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="50" t="s">
-        <v>168</v>
-      </c>
-      <c r="B22" s="50" t="s">
-        <v>173</v>
-      </c>
-      <c r="C22" s="50" t="s">
-        <v>174</v>
-      </c>
-      <c r="D22" s="50" t="s">
-        <v>62</v>
-      </c>
-      <c r="E22" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="50" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="50" t="s">
-        <v>168</v>
-      </c>
-      <c r="B23" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="C23" s="50" t="s">
-        <v>176</v>
-      </c>
-      <c r="D23" s="50" t="s">
-        <v>142</v>
-      </c>
-      <c r="E23" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="50" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="50" t="s">
-        <v>168</v>
-      </c>
-      <c r="B24" s="50" t="s">
-        <v>177</v>
-      </c>
-      <c r="C24" s="50" t="s">
-        <v>178</v>
-      </c>
-      <c r="D24" s="50" t="s">
+      <c r="E31" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="51" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="51" t="s">
+        <v>190</v>
+      </c>
+      <c r="B32" s="51" t="s">
+        <v>195</v>
+      </c>
+      <c r="C32" s="51" t="s">
+        <v>196</v>
+      </c>
+      <c r="D32" s="51" t="s">
+        <v>141</v>
+      </c>
+      <c r="E32" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="G32" s="51" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="51" t="s">
+        <v>190</v>
+      </c>
+      <c r="B33" s="51" t="s">
+        <v>197</v>
+      </c>
+      <c r="C33" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="D33" s="51" t="s">
         <v>67</v>
       </c>
-      <c r="E24" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="50" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="51" t="s">
-        <v>179</v>
-      </c>
-      <c r="B25" s="51" t="s">
-        <v>180</v>
-      </c>
-      <c r="C25" s="51" t="s">
-        <v>181</v>
-      </c>
-      <c r="D25" s="51" t="s">
-        <v>73</v>
-      </c>
-      <c r="E25" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" s="51" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="51" t="s">
-        <v>179</v>
-      </c>
-      <c r="B26" s="51" t="s">
-        <v>182</v>
-      </c>
-      <c r="C26" s="51" t="s">
-        <v>183</v>
-      </c>
-      <c r="D26" s="51" t="s">
-        <v>58</v>
-      </c>
-      <c r="E26" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="51" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="51" t="s">
-        <v>179</v>
-      </c>
-      <c r="B27" s="51" t="s">
-        <v>184</v>
-      </c>
-      <c r="C27" s="51" t="s">
-        <v>185</v>
-      </c>
-      <c r="D27" s="51" t="s">
-        <v>62</v>
-      </c>
-      <c r="E27" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="51" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="51" t="s">
-        <v>179</v>
-      </c>
-      <c r="B28" s="51" t="s">
-        <v>186</v>
-      </c>
-      <c r="C28" s="51" t="s">
-        <v>187</v>
-      </c>
-      <c r="D28" s="51" t="s">
-        <v>142</v>
-      </c>
-      <c r="E28" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="51" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="51" t="s">
-        <v>179</v>
-      </c>
-      <c r="B29" s="51" t="s">
-        <v>188</v>
-      </c>
-      <c r="C29" s="51" t="s">
-        <v>189</v>
-      </c>
-      <c r="D29" s="51" t="s">
-        <v>67</v>
-      </c>
-      <c r="E29" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="51" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="52.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="52" t="s">
-        <v>190</v>
-      </c>
-      <c r="B30" s="52" t="s">
-        <v>191</v>
-      </c>
-      <c r="C30" s="52" t="s">
-        <v>192</v>
-      </c>
-      <c r="D30" s="52" t="s">
-        <v>73</v>
-      </c>
-      <c r="E30" s="52" t="n">
-        <v>2</v>
-      </c>
-      <c r="F30" s="52" t="n">
-        <v>2</v>
-      </c>
-      <c r="G30" s="52" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="52" t="s">
-        <v>190</v>
-      </c>
-      <c r="B31" s="52" t="s">
-        <v>193</v>
-      </c>
-      <c r="C31" s="52" t="s">
-        <v>194</v>
-      </c>
-      <c r="D31" s="52" t="s">
-        <v>62</v>
-      </c>
-      <c r="E31" s="52" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" s="52" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" s="52" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="52" t="s">
-        <v>190</v>
-      </c>
-      <c r="B32" s="52" t="s">
-        <v>195</v>
-      </c>
-      <c r="C32" s="52" t="s">
-        <v>196</v>
-      </c>
-      <c r="D32" s="52" t="s">
-        <v>142</v>
-      </c>
-      <c r="E32" s="52" t="n">
-        <v>2</v>
-      </c>
-      <c r="F32" s="52" t="n">
-        <v>2</v>
-      </c>
-      <c r="G32" s="52" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="52" t="s">
-        <v>190</v>
-      </c>
-      <c r="B33" s="52" t="s">
-        <v>197</v>
-      </c>
-      <c r="C33" s="52" t="s">
-        <v>198</v>
-      </c>
-      <c r="D33" s="52" t="s">
-        <v>67</v>
-      </c>
-      <c r="E33" s="52" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="52" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" s="52" t="s">
-        <v>133</v>
+      <c r="E33" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="51" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3731,104 +3727,104 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="53" t="s">
+      <c r="B6" s="52" t="s">
         <v>205</v>
       </c>
-      <c r="C6" s="54" t="s">
+      <c r="C6" s="53" t="s">
         <v>206</v>
       </c>
-      <c r="D6" s="53" t="s">
+      <c r="D6" s="52" t="s">
         <v>207</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="53" t="s">
+      <c r="B7" s="52" t="s">
         <v>208</v>
       </c>
-      <c r="C7" s="54" t="s">
+      <c r="C7" s="53" t="s">
         <v>206</v>
       </c>
-      <c r="D7" s="53" t="s">
+      <c r="D7" s="52" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="53" t="s">
+      <c r="B8" s="52" t="s">
         <v>210</v>
       </c>
-      <c r="C8" s="54" t="s">
+      <c r="C8" s="53" t="s">
         <v>206</v>
       </c>
-      <c r="D8" s="53" t="s">
+      <c r="D8" s="52" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="53" t="s">
+      <c r="B9" s="52" t="s">
         <v>212</v>
       </c>
-      <c r="C9" s="54" t="s">
+      <c r="C9" s="53" t="s">
         <v>206</v>
       </c>
-      <c r="D9" s="53" t="s">
+      <c r="D9" s="52" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="53" t="s">
+      <c r="B10" s="52" t="s">
         <v>214</v>
       </c>
-      <c r="C10" s="54" t="s">
+      <c r="C10" s="53" t="s">
         <v>206</v>
       </c>
-      <c r="D10" s="53"/>
+      <c r="D10" s="52"/>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="53" t="s">
+      <c r="B11" s="52" t="s">
         <v>215</v>
       </c>
-      <c r="C11" s="54" t="s">
+      <c r="C11" s="53" t="s">
         <v>206</v>
       </c>
-      <c r="D11" s="53" t="s">
+      <c r="D11" s="52" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="53" t="s">
+      <c r="B12" s="52" t="s">
         <v>217</v>
       </c>
-      <c r="C12" s="54" t="s">
+      <c r="C12" s="53" t="s">
         <v>206</v>
       </c>
-      <c r="D12" s="53"/>
+      <c r="D12" s="52"/>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="53" t="s">
+      <c r="B13" s="52" t="s">
         <v>218</v>
       </c>
-      <c r="C13" s="54" t="s">
+      <c r="C13" s="53" t="s">
         <v>206</v>
       </c>
-      <c r="D13" s="53"/>
+      <c r="D13" s="52"/>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="53" t="s">
+      <c r="B14" s="52" t="s">
         <v>219</v>
       </c>
-      <c r="C14" s="54" t="s">
+      <c r="C14" s="53" t="s">
         <v>206</v>
       </c>
-      <c r="D14" s="53"/>
+      <c r="D14" s="52"/>
     </row>
     <row r="15" customFormat="false" ht="53.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="53" t="s">
+      <c r="B15" s="52" t="s">
         <v>220</v>
       </c>
-      <c r="C15" s="54" t="s">
+      <c r="C15" s="53" t="s">
         <v>206</v>
       </c>
-      <c r="D15" s="53" t="s">
+      <c r="D15" s="52" t="s">
         <v>221</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(sprint 3): mise à jour backlog Excel avec répartition sprint 3
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-09-sprint-backlog-v3.0.xlsx
+++ b/docs/cadrage/equipe-09-sprint-backlog-v3.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Garde" sheetId="1" state="visible" r:id="rId3"/>
@@ -426,7 +426,7 @@
     <t xml:space="preserve">T-03.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Setup Llama 3.1 8B en local (Ollama) + wrapper d'appel
+    <t xml:space="preserve">Setup Llama 3.2 3B en local (Ollama) + wrapper d'appel
 </t>
   </si>
   <si>
@@ -1093,7 +1093,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1263,6 +1263,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="27" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2494,16 +2498,16 @@
       <c r="C20" s="43" t="s">
         <v>132</v>
       </c>
-      <c r="D20" s="43" t="s">
+      <c r="D20" s="44" t="s">
         <v>58</v>
       </c>
-      <c r="E20" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" s="43" t="s">
+      <c r="E20" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="44" t="s">
         <v>59</v>
       </c>
     </row>
@@ -2511,22 +2515,22 @@
       <c r="A21" s="41" t="s">
         <v>130</v>
       </c>
-      <c r="B21" s="45" t="s">
+      <c r="B21" s="46" t="s">
         <v>133</v>
       </c>
       <c r="C21" s="41" t="s">
         <v>134</v>
       </c>
-      <c r="D21" s="43" t="s">
+      <c r="D21" s="44" t="s">
         <v>58</v>
       </c>
-      <c r="E21" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="43" t="s">
+      <c r="E21" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="44" t="s">
         <v>59</v>
       </c>
     </row>
@@ -2534,22 +2538,22 @@
       <c r="A22" s="41" t="s">
         <v>130</v>
       </c>
-      <c r="B22" s="45" t="s">
+      <c r="B22" s="46" t="s">
         <v>135</v>
       </c>
-      <c r="C22" s="46" t="s">
+      <c r="C22" s="47" t="s">
         <v>136</v>
       </c>
-      <c r="D22" s="43" t="s">
+      <c r="D22" s="44" t="s">
         <v>73</v>
       </c>
-      <c r="E22" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="43" t="s">
+      <c r="E22" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="44" t="s">
         <v>59</v>
       </c>
     </row>
@@ -2557,22 +2561,22 @@
       <c r="A23" s="41" t="s">
         <v>130</v>
       </c>
-      <c r="B23" s="45" t="s">
+      <c r="B23" s="46" t="s">
         <v>137</v>
       </c>
       <c r="C23" s="41" t="s">
         <v>138</v>
       </c>
-      <c r="D23" s="43" t="s">
+      <c r="D23" s="44" t="s">
         <v>62</v>
       </c>
-      <c r="E23" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="43" t="s">
+      <c r="E23" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="44" t="s">
         <v>59</v>
       </c>
     </row>
@@ -2580,22 +2584,22 @@
       <c r="A24" s="41" t="s">
         <v>130</v>
       </c>
-      <c r="B24" s="45" t="s">
+      <c r="B24" s="46" t="s">
         <v>139</v>
       </c>
-      <c r="C24" s="47" t="s">
+      <c r="C24" s="48" t="s">
         <v>140</v>
       </c>
-      <c r="D24" s="43" t="s">
+      <c r="D24" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="E24" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="43" t="s">
+      <c r="E24" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="44" t="s">
         <v>59</v>
       </c>
     </row>
@@ -2603,137 +2607,137 @@
       <c r="A25" s="41" t="s">
         <v>130</v>
       </c>
-      <c r="B25" s="45" t="s">
+      <c r="B25" s="46" t="s">
         <v>142</v>
       </c>
       <c r="C25" s="41" t="s">
         <v>143</v>
       </c>
-      <c r="D25" s="43" t="s">
+      <c r="D25" s="44" t="s">
         <v>67</v>
       </c>
-      <c r="E25" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" s="43" t="s">
+      <c r="E25" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="44" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="48" t="s">
+      <c r="A26" s="49" t="s">
         <v>144</v>
       </c>
-      <c r="B26" s="48" t="s">
+      <c r="B26" s="49" t="s">
         <v>145</v>
       </c>
-      <c r="C26" s="48" t="s">
+      <c r="C26" s="49" t="s">
         <v>146</v>
       </c>
-      <c r="D26" s="48" t="s">
+      <c r="D26" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="E26" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="43" t="s">
+      <c r="E26" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="44" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="48" t="s">
+      <c r="A27" s="49" t="s">
         <v>144</v>
       </c>
-      <c r="B27" s="48" t="s">
+      <c r="B27" s="49" t="s">
         <v>147</v>
       </c>
-      <c r="C27" s="48" t="s">
+      <c r="C27" s="49" t="s">
         <v>148</v>
       </c>
-      <c r="D27" s="48" t="s">
+      <c r="D27" s="49" t="s">
         <v>73</v>
       </c>
-      <c r="E27" s="48" t="n">
+      <c r="E27" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="F27" s="48" t="n">
+      <c r="F27" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="G27" s="43" t="s">
+      <c r="G27" s="44" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="48" t="s">
+      <c r="A28" s="49" t="s">
         <v>144</v>
       </c>
-      <c r="B28" s="48" t="s">
+      <c r="B28" s="49" t="s">
         <v>149</v>
       </c>
-      <c r="C28" s="48" t="s">
+      <c r="C28" s="49" t="s">
         <v>150</v>
       </c>
-      <c r="D28" s="48" t="s">
+      <c r="D28" s="49" t="s">
         <v>62</v>
       </c>
-      <c r="E28" s="48" t="n">
+      <c r="E28" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="F28" s="48" t="n">
+      <c r="F28" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="43" t="s">
+      <c r="G28" s="44" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="48" t="s">
+      <c r="A29" s="49" t="s">
         <v>144</v>
       </c>
-      <c r="B29" s="48" t="s">
+      <c r="B29" s="49" t="s">
         <v>151</v>
       </c>
-      <c r="C29" s="48" t="s">
+      <c r="C29" s="49" t="s">
         <v>152</v>
       </c>
-      <c r="D29" s="48" t="s">
+      <c r="D29" s="49" t="s">
         <v>141</v>
       </c>
-      <c r="E29" s="48" t="n">
+      <c r="E29" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="F29" s="48" t="n">
+      <c r="F29" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="G29" s="43" t="s">
+      <c r="G29" s="44" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="48" t="s">
+      <c r="A30" s="49" t="s">
         <v>144</v>
       </c>
-      <c r="B30" s="48" t="s">
+      <c r="B30" s="49" t="s">
         <v>153</v>
       </c>
-      <c r="C30" s="48" t="s">
+      <c r="C30" s="49" t="s">
         <v>154</v>
       </c>
-      <c r="D30" s="48" t="s">
+      <c r="D30" s="49" t="s">
         <v>67</v>
       </c>
-      <c r="E30" s="48" t="n">
+      <c r="E30" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="F30" s="48" t="n">
+      <c r="F30" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="G30" s="43" t="s">
+      <c r="G30" s="44" t="s">
         <v>59</v>
       </c>
     </row>
@@ -3129,324 +3133,324 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="45.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="49" t="s">
+      <c r="A20" s="50" t="s">
         <v>167</v>
       </c>
-      <c r="B20" s="49" t="s">
+      <c r="B20" s="50" t="s">
         <v>168</v>
       </c>
-      <c r="C20" s="49" t="s">
+      <c r="C20" s="50" t="s">
         <v>169</v>
       </c>
-      <c r="D20" s="49" t="s">
+      <c r="D20" s="50" t="s">
         <v>58</v>
       </c>
-      <c r="E20" s="49" t="n">
+      <c r="E20" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="F20" s="49" t="n">
+      <c r="F20" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="G20" s="49" t="s">
+      <c r="G20" s="50" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="49" t="s">
+      <c r="A21" s="50" t="s">
         <v>167</v>
       </c>
-      <c r="B21" s="49" t="s">
+      <c r="B21" s="50" t="s">
         <v>171</v>
       </c>
-      <c r="C21" s="49" t="s">
+      <c r="C21" s="50" t="s">
         <v>172</v>
       </c>
-      <c r="D21" s="49" t="s">
+      <c r="D21" s="50" t="s">
         <v>62</v>
       </c>
-      <c r="E21" s="49" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="49" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="49" t="s">
+      <c r="E21" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="50" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="49" t="s">
+      <c r="A22" s="50" t="s">
         <v>167</v>
       </c>
-      <c r="B22" s="49" t="s">
+      <c r="B22" s="50" t="s">
         <v>173</v>
       </c>
-      <c r="C22" s="49" t="s">
+      <c r="C22" s="50" t="s">
         <v>174</v>
       </c>
-      <c r="D22" s="49" t="s">
+      <c r="D22" s="50" t="s">
         <v>62</v>
       </c>
-      <c r="E22" s="49" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="49" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="49" t="s">
+      <c r="E22" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="50" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="49" t="s">
+      <c r="A23" s="50" t="s">
         <v>167</v>
       </c>
-      <c r="B23" s="49" t="s">
+      <c r="B23" s="50" t="s">
         <v>175</v>
       </c>
-      <c r="C23" s="49" t="s">
+      <c r="C23" s="50" t="s">
         <v>176</v>
       </c>
-      <c r="D23" s="49" t="s">
+      <c r="D23" s="50" t="s">
         <v>141</v>
       </c>
-      <c r="E23" s="49" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="49" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="49" t="s">
+      <c r="E23" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="50" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="49" t="s">
+      <c r="A24" s="50" t="s">
         <v>167</v>
       </c>
-      <c r="B24" s="49" t="s">
+      <c r="B24" s="50" t="s">
         <v>177</v>
       </c>
-      <c r="C24" s="49" t="s">
+      <c r="C24" s="50" t="s">
         <v>178</v>
       </c>
-      <c r="D24" s="49" t="s">
+      <c r="D24" s="50" t="s">
         <v>67</v>
       </c>
-      <c r="E24" s="49" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="49" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="49" t="s">
+      <c r="E24" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="50" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="50" t="s">
+      <c r="A25" s="51" t="s">
         <v>179</v>
       </c>
-      <c r="B25" s="50" t="s">
+      <c r="B25" s="51" t="s">
         <v>180</v>
       </c>
-      <c r="C25" s="50" t="s">
+      <c r="C25" s="51" t="s">
         <v>181</v>
       </c>
-      <c r="D25" s="50" t="s">
+      <c r="D25" s="51" t="s">
         <v>73</v>
       </c>
-      <c r="E25" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" s="50" t="s">
+      <c r="E25" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="51" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="50" t="s">
+      <c r="A26" s="51" t="s">
         <v>179</v>
       </c>
-      <c r="B26" s="50" t="s">
+      <c r="B26" s="51" t="s">
         <v>182</v>
       </c>
-      <c r="C26" s="50" t="s">
+      <c r="C26" s="51" t="s">
         <v>183</v>
       </c>
-      <c r="D26" s="50" t="s">
+      <c r="D26" s="51" t="s">
         <v>58</v>
       </c>
-      <c r="E26" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="50" t="s">
+      <c r="E26" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="51" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="50" t="s">
+      <c r="A27" s="51" t="s">
         <v>179</v>
       </c>
-      <c r="B27" s="50" t="s">
+      <c r="B27" s="51" t="s">
         <v>184</v>
       </c>
-      <c r="C27" s="50" t="s">
+      <c r="C27" s="51" t="s">
         <v>185</v>
       </c>
-      <c r="D27" s="50" t="s">
+      <c r="D27" s="51" t="s">
         <v>62</v>
       </c>
-      <c r="E27" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="50" t="s">
+      <c r="E27" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="51" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="51" t="s">
         <v>179</v>
       </c>
-      <c r="B28" s="50" t="s">
+      <c r="B28" s="51" t="s">
         <v>186</v>
       </c>
-      <c r="C28" s="50" t="s">
+      <c r="C28" s="51" t="s">
         <v>187</v>
       </c>
-      <c r="D28" s="50" t="s">
+      <c r="D28" s="51" t="s">
         <v>141</v>
       </c>
-      <c r="E28" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="50" t="s">
+      <c r="E28" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="51" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="50" t="s">
+      <c r="A29" s="51" t="s">
         <v>179</v>
       </c>
-      <c r="B29" s="50" t="s">
+      <c r="B29" s="51" t="s">
         <v>188</v>
       </c>
-      <c r="C29" s="50" t="s">
+      <c r="C29" s="51" t="s">
         <v>189</v>
       </c>
-      <c r="D29" s="50" t="s">
+      <c r="D29" s="51" t="s">
         <v>67</v>
       </c>
-      <c r="E29" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="50" t="s">
+      <c r="E29" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="51" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="52.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="51" t="s">
+      <c r="A30" s="52" t="s">
         <v>190</v>
       </c>
-      <c r="B30" s="51" t="s">
+      <c r="B30" s="52" t="s">
         <v>191</v>
       </c>
-      <c r="C30" s="51" t="s">
+      <c r="C30" s="52" t="s">
         <v>192</v>
       </c>
-      <c r="D30" s="51" t="s">
+      <c r="D30" s="52" t="s">
         <v>73</v>
       </c>
-      <c r="E30" s="51" t="n">
+      <c r="E30" s="52" t="n">
         <v>2</v>
       </c>
-      <c r="F30" s="51" t="n">
+      <c r="F30" s="52" t="n">
         <v>2</v>
       </c>
-      <c r="G30" s="51" t="s">
+      <c r="G30" s="52" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="51" t="s">
+      <c r="A31" s="52" t="s">
         <v>190</v>
       </c>
-      <c r="B31" s="51" t="s">
+      <c r="B31" s="52" t="s">
         <v>193</v>
       </c>
-      <c r="C31" s="51" t="s">
+      <c r="C31" s="52" t="s">
         <v>194</v>
       </c>
-      <c r="D31" s="51" t="s">
+      <c r="D31" s="52" t="s">
         <v>62</v>
       </c>
-      <c r="E31" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" s="51" t="s">
+      <c r="E31" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="52" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="51" t="s">
+      <c r="A32" s="52" t="s">
         <v>190</v>
       </c>
-      <c r="B32" s="51" t="s">
+      <c r="B32" s="52" t="s">
         <v>195</v>
       </c>
-      <c r="C32" s="51" t="s">
+      <c r="C32" s="52" t="s">
         <v>196</v>
       </c>
-      <c r="D32" s="51" t="s">
+      <c r="D32" s="52" t="s">
         <v>141</v>
       </c>
-      <c r="E32" s="51" t="n">
+      <c r="E32" s="52" t="n">
         <v>2</v>
       </c>
-      <c r="F32" s="51" t="n">
+      <c r="F32" s="52" t="n">
         <v>2</v>
       </c>
-      <c r="G32" s="51" t="s">
+      <c r="G32" s="52" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="51" t="s">
+      <c r="A33" s="52" t="s">
         <v>190</v>
       </c>
-      <c r="B33" s="51" t="s">
+      <c r="B33" s="52" t="s">
         <v>197</v>
       </c>
-      <c r="C33" s="51" t="s">
+      <c r="C33" s="52" t="s">
         <v>198</v>
       </c>
-      <c r="D33" s="51" t="s">
+      <c r="D33" s="52" t="s">
         <v>67</v>
       </c>
-      <c r="E33" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" s="51" t="s">
+      <c r="E33" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="52" t="s">
         <v>170</v>
       </c>
     </row>
@@ -3727,104 +3731,104 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="52" t="s">
+      <c r="B6" s="53" t="s">
         <v>205</v>
       </c>
-      <c r="C6" s="53" t="s">
+      <c r="C6" s="54" t="s">
         <v>206</v>
       </c>
-      <c r="D6" s="52" t="s">
+      <c r="D6" s="53" t="s">
         <v>207</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="52" t="s">
+      <c r="B7" s="53" t="s">
         <v>208</v>
       </c>
-      <c r="C7" s="53" t="s">
+      <c r="C7" s="54" t="s">
         <v>206</v>
       </c>
-      <c r="D7" s="52" t="s">
+      <c r="D7" s="53" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="52" t="s">
+      <c r="B8" s="53" t="s">
         <v>210</v>
       </c>
-      <c r="C8" s="53" t="s">
+      <c r="C8" s="54" t="s">
         <v>206</v>
       </c>
-      <c r="D8" s="52" t="s">
+      <c r="D8" s="53" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="52" t="s">
+      <c r="B9" s="53" t="s">
         <v>212</v>
       </c>
-      <c r="C9" s="53" t="s">
+      <c r="C9" s="54" t="s">
         <v>206</v>
       </c>
-      <c r="D9" s="52" t="s">
+      <c r="D9" s="53" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="52" t="s">
+      <c r="B10" s="53" t="s">
         <v>214</v>
       </c>
-      <c r="C10" s="53" t="s">
+      <c r="C10" s="54" t="s">
         <v>206</v>
       </c>
-      <c r="D10" s="52"/>
+      <c r="D10" s="53"/>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="52" t="s">
+      <c r="B11" s="53" t="s">
         <v>215</v>
       </c>
-      <c r="C11" s="53" t="s">
+      <c r="C11" s="54" t="s">
         <v>206</v>
       </c>
-      <c r="D11" s="52" t="s">
+      <c r="D11" s="53" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="52" t="s">
+      <c r="B12" s="53" t="s">
         <v>217</v>
       </c>
-      <c r="C12" s="53" t="s">
+      <c r="C12" s="54" t="s">
         <v>206</v>
       </c>
-      <c r="D12" s="52"/>
+      <c r="D12" s="53"/>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="52" t="s">
+      <c r="B13" s="53" t="s">
         <v>218</v>
       </c>
-      <c r="C13" s="53" t="s">
+      <c r="C13" s="54" t="s">
         <v>206</v>
       </c>
-      <c r="D13" s="52"/>
+      <c r="D13" s="53"/>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="52" t="s">
+      <c r="B14" s="53" t="s">
         <v>219</v>
       </c>
-      <c r="C14" s="53" t="s">
+      <c r="C14" s="54" t="s">
         <v>206</v>
       </c>
-      <c r="D14" s="52"/>
+      <c r="D14" s="53"/>
     </row>
     <row r="15" customFormat="false" ht="53.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="52" t="s">
+      <c r="B15" s="53" t="s">
         <v>220</v>
       </c>
-      <c r="C15" s="53" t="s">
+      <c r="C15" s="54" t="s">
         <v>206</v>
       </c>
-      <c r="D15" s="52" t="s">
+      <c r="D15" s="53" t="s">
         <v>221</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(fix): temps restant 0
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-09-sprint-backlog-v3.0.xlsx
+++ b/docs/cadrage/equipe-09-sprint-backlog-v3.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Garde" sheetId="1" state="visible" r:id="rId3"/>
@@ -1093,7 +1093,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="53">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1254,10 +1254,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="21" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1271,10 +1267,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1294,15 +1286,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="29" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="29" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="29" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2413,7 +2405,7 @@
       <c r="A10" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="40" t="s">
+      <c r="B10" s="20" t="s">
         <v>127</v>
       </c>
     </row>
@@ -2489,255 +2481,255 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="41" t="s">
+      <c r="A20" s="40" t="s">
         <v>130</v>
       </c>
-      <c r="B20" s="42" t="s">
+      <c r="B20" s="41" t="s">
         <v>131</v>
       </c>
-      <c r="C20" s="43" t="s">
+      <c r="C20" s="42" t="s">
         <v>132</v>
       </c>
-      <c r="D20" s="44" t="s">
+      <c r="D20" s="42" t="s">
         <v>58</v>
       </c>
-      <c r="E20" s="45" t="n">
+      <c r="E20" s="43" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="45" t="n">
+      <c r="F20" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="42" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="B21" s="44" t="s">
+        <v>133</v>
+      </c>
+      <c r="C21" s="40" t="s">
+        <v>134</v>
+      </c>
+      <c r="D21" s="42" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" s="43" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="44" t="s">
+      <c r="F21" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="42" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="41" t="s">
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="40" t="s">
         <v>130</v>
       </c>
-      <c r="B21" s="46" t="s">
-        <v>133</v>
-      </c>
-      <c r="C21" s="41" t="s">
-        <v>134</v>
-      </c>
-      <c r="D21" s="44" t="s">
+      <c r="B22" s="44" t="s">
+        <v>135</v>
+      </c>
+      <c r="C22" s="45" t="s">
+        <v>136</v>
+      </c>
+      <c r="D22" s="42" t="s">
+        <v>73</v>
+      </c>
+      <c r="E22" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="42" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="B23" s="44" t="s">
+        <v>137</v>
+      </c>
+      <c r="C23" s="40" t="s">
+        <v>138</v>
+      </c>
+      <c r="D23" s="42" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="42" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="B24" s="44" t="s">
+        <v>139</v>
+      </c>
+      <c r="C24" s="46" t="s">
+        <v>140</v>
+      </c>
+      <c r="D24" s="42" t="s">
+        <v>141</v>
+      </c>
+      <c r="E24" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="42" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="B25" s="44" t="s">
+        <v>142</v>
+      </c>
+      <c r="C25" s="40" t="s">
+        <v>143</v>
+      </c>
+      <c r="D25" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="E25" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="42" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="47" t="s">
+        <v>144</v>
+      </c>
+      <c r="B26" s="47" t="s">
+        <v>145</v>
+      </c>
+      <c r="C26" s="47" t="s">
+        <v>146</v>
+      </c>
+      <c r="D26" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="E21" s="45" t="n">
+      <c r="E26" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="F21" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="44" t="s">
+      <c r="F26" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="42" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="41" t="s">
-        <v>130</v>
-      </c>
-      <c r="B22" s="46" t="s">
-        <v>135</v>
-      </c>
-      <c r="C22" s="47" t="s">
-        <v>136</v>
-      </c>
-      <c r="D22" s="44" t="s">
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="47" t="s">
+        <v>144</v>
+      </c>
+      <c r="B27" s="47" t="s">
+        <v>147</v>
+      </c>
+      <c r="C27" s="47" t="s">
+        <v>148</v>
+      </c>
+      <c r="D27" s="47" t="s">
         <v>73</v>
       </c>
-      <c r="E22" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="44" t="s">
+      <c r="E27" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="42" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="41" t="s">
-        <v>130</v>
-      </c>
-      <c r="B23" s="46" t="s">
-        <v>137</v>
-      </c>
-      <c r="C23" s="41" t="s">
-        <v>138</v>
-      </c>
-      <c r="D23" s="44" t="s">
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="47" t="s">
+        <v>144</v>
+      </c>
+      <c r="B28" s="47" t="s">
+        <v>149</v>
+      </c>
+      <c r="C28" s="47" t="s">
+        <v>150</v>
+      </c>
+      <c r="D28" s="47" t="s">
         <v>62</v>
       </c>
-      <c r="E23" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="44" t="s">
+      <c r="E28" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="42" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="41" t="s">
-        <v>130</v>
-      </c>
-      <c r="B24" s="46" t="s">
-        <v>139</v>
-      </c>
-      <c r="C24" s="48" t="s">
-        <v>140</v>
-      </c>
-      <c r="D24" s="44" t="s">
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="47" t="s">
+        <v>144</v>
+      </c>
+      <c r="B29" s="47" t="s">
+        <v>151</v>
+      </c>
+      <c r="C29" s="47" t="s">
+        <v>152</v>
+      </c>
+      <c r="D29" s="47" t="s">
         <v>141</v>
       </c>
-      <c r="E24" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="44" t="s">
+      <c r="E29" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="42" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="41" t="s">
-        <v>130</v>
-      </c>
-      <c r="B25" s="46" t="s">
-        <v>142</v>
-      </c>
-      <c r="C25" s="41" t="s">
-        <v>143</v>
-      </c>
-      <c r="D25" s="44" t="s">
+    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="47" t="s">
+        <v>144</v>
+      </c>
+      <c r="B30" s="47" t="s">
+        <v>153</v>
+      </c>
+      <c r="C30" s="47" t="s">
+        <v>154</v>
+      </c>
+      <c r="D30" s="47" t="s">
         <v>67</v>
       </c>
-      <c r="E25" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="45" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" s="44" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="49" t="s">
-        <v>144</v>
-      </c>
-      <c r="B26" s="49" t="s">
-        <v>145</v>
-      </c>
-      <c r="C26" s="49" t="s">
-        <v>146</v>
-      </c>
-      <c r="D26" s="49" t="s">
-        <v>58</v>
-      </c>
-      <c r="E26" s="49" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="49" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="44" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="49" t="s">
-        <v>144</v>
-      </c>
-      <c r="B27" s="49" t="s">
-        <v>147</v>
-      </c>
-      <c r="C27" s="49" t="s">
-        <v>148</v>
-      </c>
-      <c r="D27" s="49" t="s">
-        <v>73</v>
-      </c>
-      <c r="E27" s="49" t="n">
+      <c r="E30" s="47" t="n">
         <v>2</v>
       </c>
-      <c r="F27" s="49" t="n">
-        <v>2</v>
-      </c>
-      <c r="G27" s="44" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="49" t="s">
-        <v>144</v>
-      </c>
-      <c r="B28" s="49" t="s">
-        <v>149</v>
-      </c>
-      <c r="C28" s="49" t="s">
-        <v>150</v>
-      </c>
-      <c r="D28" s="49" t="s">
-        <v>62</v>
-      </c>
-      <c r="E28" s="49" t="n">
-        <v>2</v>
-      </c>
-      <c r="F28" s="49" t="n">
-        <v>2</v>
-      </c>
-      <c r="G28" s="44" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="49" t="s">
-        <v>144</v>
-      </c>
-      <c r="B29" s="49" t="s">
-        <v>151</v>
-      </c>
-      <c r="C29" s="49" t="s">
-        <v>152</v>
-      </c>
-      <c r="D29" s="49" t="s">
-        <v>141</v>
-      </c>
-      <c r="E29" s="49" t="n">
-        <v>2</v>
-      </c>
-      <c r="F29" s="49" t="n">
-        <v>2</v>
-      </c>
-      <c r="G29" s="44" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="49" t="s">
-        <v>144</v>
-      </c>
-      <c r="B30" s="49" t="s">
-        <v>153</v>
-      </c>
-      <c r="C30" s="49" t="s">
-        <v>154</v>
-      </c>
-      <c r="D30" s="49" t="s">
-        <v>67</v>
-      </c>
-      <c r="E30" s="49" t="n">
-        <v>2</v>
-      </c>
-      <c r="F30" s="49" t="n">
-        <v>2</v>
-      </c>
-      <c r="G30" s="44" t="s">
+      <c r="F30" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="42" t="s">
         <v>59</v>
       </c>
     </row>
@@ -2752,7 +2744,7 @@
         <v>15</v>
       </c>
       <c r="F31" s="33" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G31" s="34"/>
     </row>
@@ -3133,328 +3125,328 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="45.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="48" t="s">
         <v>167</v>
       </c>
-      <c r="B20" s="50" t="s">
+      <c r="B20" s="48" t="s">
         <v>168</v>
       </c>
-      <c r="C20" s="50" t="s">
+      <c r="C20" s="48" t="s">
         <v>169</v>
       </c>
-      <c r="D20" s="50" t="s">
+      <c r="D20" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="E20" s="50" t="n">
+      <c r="E20" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="F20" s="50" t="n">
+      <c r="F20" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="G20" s="50" t="s">
+      <c r="G20" s="48" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="50" t="s">
+      <c r="A21" s="48" t="s">
         <v>167</v>
       </c>
-      <c r="B21" s="50" t="s">
+      <c r="B21" s="48" t="s">
         <v>171</v>
       </c>
-      <c r="C21" s="50" t="s">
+      <c r="C21" s="48" t="s">
         <v>172</v>
       </c>
-      <c r="D21" s="50" t="s">
+      <c r="D21" s="48" t="s">
         <v>62</v>
       </c>
-      <c r="E21" s="50" t="n">
+      <c r="E21" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="F21" s="50" t="n">
+      <c r="F21" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="G21" s="50" t="s">
+      <c r="G21" s="48" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="50" t="s">
+      <c r="A22" s="48" t="s">
         <v>167</v>
       </c>
-      <c r="B22" s="50" t="s">
+      <c r="B22" s="48" t="s">
         <v>173</v>
       </c>
-      <c r="C22" s="50" t="s">
+      <c r="C22" s="48" t="s">
         <v>174</v>
       </c>
-      <c r="D22" s="50" t="s">
+      <c r="D22" s="48" t="s">
         <v>62</v>
       </c>
-      <c r="E22" s="50" t="n">
+      <c r="E22" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="F22" s="50" t="n">
+      <c r="F22" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="50" t="s">
+      <c r="G22" s="48" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="48" t="s">
         <v>167</v>
       </c>
-      <c r="B23" s="50" t="s">
+      <c r="B23" s="48" t="s">
         <v>175</v>
       </c>
-      <c r="C23" s="50" t="s">
+      <c r="C23" s="48" t="s">
         <v>176</v>
       </c>
-      <c r="D23" s="50" t="s">
+      <c r="D23" s="48" t="s">
         <v>141</v>
       </c>
-      <c r="E23" s="50" t="n">
+      <c r="E23" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="F23" s="50" t="n">
+      <c r="F23" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="50" t="s">
+      <c r="G23" s="48" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="50" t="s">
+      <c r="A24" s="48" t="s">
         <v>167</v>
       </c>
-      <c r="B24" s="50" t="s">
+      <c r="B24" s="48" t="s">
         <v>177</v>
       </c>
-      <c r="C24" s="50" t="s">
+      <c r="C24" s="48" t="s">
         <v>178</v>
       </c>
-      <c r="D24" s="50" t="s">
+      <c r="D24" s="48" t="s">
         <v>67</v>
       </c>
-      <c r="E24" s="50" t="n">
+      <c r="E24" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="F24" s="50" t="n">
+      <c r="F24" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="G24" s="50" t="s">
+      <c r="G24" s="48" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="51" t="s">
+      <c r="A25" s="49" t="s">
         <v>179</v>
       </c>
-      <c r="B25" s="51" t="s">
+      <c r="B25" s="49" t="s">
         <v>180</v>
       </c>
-      <c r="C25" s="51" t="s">
+      <c r="C25" s="49" t="s">
         <v>181</v>
       </c>
-      <c r="D25" s="51" t="s">
+      <c r="D25" s="49" t="s">
         <v>73</v>
       </c>
-      <c r="E25" s="51" t="n">
+      <c r="E25" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="F25" s="51" t="n">
+      <c r="F25" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="G25" s="51" t="s">
+      <c r="G25" s="49" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="51" t="s">
+      <c r="A26" s="49" t="s">
         <v>179</v>
       </c>
-      <c r="B26" s="51" t="s">
+      <c r="B26" s="49" t="s">
         <v>182</v>
       </c>
-      <c r="C26" s="51" t="s">
+      <c r="C26" s="49" t="s">
         <v>183</v>
       </c>
-      <c r="D26" s="51" t="s">
+      <c r="D26" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="E26" s="51" t="n">
+      <c r="E26" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="F26" s="51" t="n">
+      <c r="F26" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="G26" s="51" t="s">
+      <c r="G26" s="49" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="51" t="s">
+      <c r="A27" s="49" t="s">
         <v>179</v>
       </c>
-      <c r="B27" s="51" t="s">
+      <c r="B27" s="49" t="s">
         <v>184</v>
       </c>
-      <c r="C27" s="51" t="s">
+      <c r="C27" s="49" t="s">
         <v>185</v>
       </c>
-      <c r="D27" s="51" t="s">
+      <c r="D27" s="49" t="s">
         <v>62</v>
       </c>
-      <c r="E27" s="51" t="n">
+      <c r="E27" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="F27" s="51" t="n">
+      <c r="F27" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="G27" s="51" t="s">
+      <c r="G27" s="49" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="51" t="s">
+      <c r="A28" s="49" t="s">
         <v>179</v>
       </c>
-      <c r="B28" s="51" t="s">
+      <c r="B28" s="49" t="s">
         <v>186</v>
       </c>
-      <c r="C28" s="51" t="s">
+      <c r="C28" s="49" t="s">
         <v>187</v>
       </c>
-      <c r="D28" s="51" t="s">
+      <c r="D28" s="49" t="s">
         <v>141</v>
       </c>
-      <c r="E28" s="51" t="n">
+      <c r="E28" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="F28" s="51" t="n">
+      <c r="F28" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="G28" s="51" t="s">
+      <c r="G28" s="49" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="51" t="s">
+      <c r="A29" s="49" t="s">
         <v>179</v>
       </c>
-      <c r="B29" s="51" t="s">
+      <c r="B29" s="49" t="s">
         <v>188</v>
       </c>
-      <c r="C29" s="51" t="s">
+      <c r="C29" s="49" t="s">
         <v>189</v>
       </c>
-      <c r="D29" s="51" t="s">
+      <c r="D29" s="49" t="s">
         <v>67</v>
       </c>
-      <c r="E29" s="51" t="n">
+      <c r="E29" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="F29" s="51" t="n">
+      <c r="F29" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="51" t="s">
+      <c r="G29" s="49" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="52.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="52" t="s">
+      <c r="A30" s="50" t="s">
         <v>190</v>
       </c>
-      <c r="B30" s="52" t="s">
+      <c r="B30" s="50" t="s">
         <v>191</v>
       </c>
-      <c r="C30" s="52" t="s">
+      <c r="C30" s="50" t="s">
         <v>192</v>
       </c>
-      <c r="D30" s="52" t="s">
+      <c r="D30" s="50" t="s">
         <v>73</v>
       </c>
-      <c r="E30" s="52" t="n">
+      <c r="E30" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="F30" s="52" t="n">
+      <c r="F30" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="G30" s="52" t="s">
+      <c r="G30" s="50" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="52" t="s">
+      <c r="A31" s="50" t="s">
         <v>190</v>
       </c>
-      <c r="B31" s="52" t="s">
+      <c r="B31" s="50" t="s">
         <v>193</v>
       </c>
-      <c r="C31" s="52" t="s">
+      <c r="C31" s="50" t="s">
         <v>194</v>
       </c>
-      <c r="D31" s="52" t="s">
+      <c r="D31" s="50" t="s">
         <v>62</v>
       </c>
-      <c r="E31" s="52" t="n">
+      <c r="E31" s="50" t="n">
         <v>1</v>
       </c>
-      <c r="F31" s="52" t="n">
+      <c r="F31" s="50" t="n">
         <v>1</v>
       </c>
-      <c r="G31" s="52" t="s">
+      <c r="G31" s="50" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="52" t="s">
+      <c r="A32" s="50" t="s">
         <v>190</v>
       </c>
-      <c r="B32" s="52" t="s">
+      <c r="B32" s="50" t="s">
         <v>195</v>
       </c>
-      <c r="C32" s="52" t="s">
+      <c r="C32" s="50" t="s">
         <v>196</v>
       </c>
-      <c r="D32" s="52" t="s">
+      <c r="D32" s="50" t="s">
         <v>141</v>
       </c>
-      <c r="E32" s="52" t="n">
+      <c r="E32" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="F32" s="52" t="n">
+      <c r="F32" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="G32" s="52" t="s">
+      <c r="G32" s="50" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="52" t="s">
+      <c r="A33" s="50" t="s">
         <v>190</v>
       </c>
-      <c r="B33" s="52" t="s">
+      <c r="B33" s="50" t="s">
         <v>197</v>
       </c>
-      <c r="C33" s="52" t="s">
+      <c r="C33" s="50" t="s">
         <v>198</v>
       </c>
-      <c r="D33" s="52" t="s">
+      <c r="D33" s="50" t="s">
         <v>67</v>
       </c>
-      <c r="E33" s="52" t="n">
+      <c r="E33" s="50" t="n">
         <v>1</v>
       </c>
-      <c r="F33" s="52" t="n">
+      <c r="F33" s="50" t="n">
         <v>1</v>
       </c>
-      <c r="G33" s="52" t="s">
+      <c r="G33" s="50" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="33" t="s">
         <v>82</v>
       </c>
@@ -3731,104 +3723,104 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="53" t="s">
+      <c r="B6" s="51" t="s">
         <v>205</v>
       </c>
-      <c r="C6" s="54" t="s">
+      <c r="C6" s="52" t="s">
         <v>206</v>
       </c>
-      <c r="D6" s="53" t="s">
+      <c r="D6" s="51" t="s">
         <v>207</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="53" t="s">
+      <c r="B7" s="51" t="s">
         <v>208</v>
       </c>
-      <c r="C7" s="54" t="s">
+      <c r="C7" s="52" t="s">
         <v>206</v>
       </c>
-      <c r="D7" s="53" t="s">
+      <c r="D7" s="51" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="53" t="s">
+      <c r="B8" s="51" t="s">
         <v>210</v>
       </c>
-      <c r="C8" s="54" t="s">
+      <c r="C8" s="52" t="s">
         <v>206</v>
       </c>
-      <c r="D8" s="53" t="s">
+      <c r="D8" s="51" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="53" t="s">
+      <c r="B9" s="51" t="s">
         <v>212</v>
       </c>
-      <c r="C9" s="54" t="s">
+      <c r="C9" s="52" t="s">
         <v>206</v>
       </c>
-      <c r="D9" s="53" t="s">
+      <c r="D9" s="51" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="53" t="s">
+      <c r="B10" s="51" t="s">
         <v>214</v>
       </c>
-      <c r="C10" s="54" t="s">
+      <c r="C10" s="52" t="s">
         <v>206</v>
       </c>
-      <c r="D10" s="53"/>
+      <c r="D10" s="51"/>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="53" t="s">
+      <c r="B11" s="51" t="s">
         <v>215</v>
       </c>
-      <c r="C11" s="54" t="s">
+      <c r="C11" s="52" t="s">
         <v>206</v>
       </c>
-      <c r="D11" s="53" t="s">
+      <c r="D11" s="51" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="53" t="s">
+      <c r="B12" s="51" t="s">
         <v>217</v>
       </c>
-      <c r="C12" s="54" t="s">
+      <c r="C12" s="52" t="s">
         <v>206</v>
       </c>
-      <c r="D12" s="53"/>
+      <c r="D12" s="51"/>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="53" t="s">
+      <c r="B13" s="51" t="s">
         <v>218</v>
       </c>
-      <c r="C13" s="54" t="s">
+      <c r="C13" s="52" t="s">
         <v>206</v>
       </c>
-      <c r="D13" s="53"/>
+      <c r="D13" s="51"/>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="53" t="s">
+      <c r="B14" s="51" t="s">
         <v>219</v>
       </c>
-      <c r="C14" s="54" t="s">
+      <c r="C14" s="52" t="s">
         <v>206</v>
       </c>
-      <c r="D14" s="53"/>
+      <c r="D14" s="51"/>
     </row>
     <row r="15" customFormat="false" ht="53.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="53" t="s">
+      <c r="B15" s="51" t="s">
         <v>220</v>
       </c>
-      <c r="C15" s="54" t="s">
+      <c r="C15" s="52" t="s">
         <v>206</v>
       </c>
-      <c r="D15" s="53" t="s">
+      <c r="D15" s="51" t="s">
         <v>221</v>
       </c>
     </row>

</xml_diff>